<commit_message>
fix(Diag): suspend charger and stop PWM gates during flash save
A page erase stalls the whole CPU ~20..40 ms on this single-bank
part; the NVM and CalLut saves already forbid switching inside that
blind window, but the Diag save (about every 60 s while charging)
did not. SaveNow runs in the control task - the context that owns
charger evaluation - so it now sets the charger suspension flag and
stops both gates synchronously around WriteFlash, then clears the
flag; duty mirrors stay untouched and the next control pass resumes
regulation seamlessly. README and validation sheet updated.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Firmware/Modules/Diag/Diag_Validation.xlsx
+++ b/Firmware/Modules/Diag/Diag_Validation.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -794,6 +794,33 @@
       <c r="E12" t="inlineStr">
         <is>
           <t>هاست 2026-10-15: ctrl از 2264/1024 (221%) به 384/1024 (37.5%) رسید و FREE RAM به 1544 بایت؛ تست برد در انتظار</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ذخیره فلش حین شارژ فعال: تعلیق شارژر دور نوشتن</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>شارژ فعال؛ صبر تا ذخیره دوره‌ای Diag؛ مشاهده گیت‌های PWM روی اسکوپ و ادامه شارژ بعد از ذخیره</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>حین پاک/نوشتن فلش هر دو گیت PWM متوقف، بعد از ذخیره شارژ بدون پرش ادامه یابد و رکورد سالم ذخیره شود</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>هاست: هر دو گیت سبز و بودجه RAM/استک سالم (ctrl ‏384/1024‎، آزاد 1544 بایت)؛ نتیجه برد: در انتظار</t>
         </is>
       </c>
     </row>
@@ -858,7 +885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -892,6 +919,23 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>رزرو هیپ لینکر صفر شد (تخصیص فقط استاتیک است) و Init/SaveNow با بافر کمکی Stage بازنویسی شدند: فقط seqها اسکالر می‌مانند؛ کامیت‌های fix(linker) و fix(Diag) روی شاخه arena/859ce091-changeover</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ممیزی خط‌به‌خط: ذخیره فلش Diag (حین شارژ حدود هر ۶۰ ثانیه) برخلاف ذخیره‌های NVM و CalLut شارژر را معلق نمی‌کرد؛ پاک‌کردن صفحه کل CPU را ۲۰ تا ۴۰ میلی‌ثانیه نگه می‌دارد و گیت‌ها داخل پنجره کور سوییچ می‌کردند</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>در func__Diag_SaveNow دور WriteFlash، ‏func__Charger_SetSuspended(true)‎ + ‏func__BspPwm_StopAll()‎ و بعد ‏SetSuspended(false)‎ اضافه شد (زمینه تسک کنترل، توقف بی‌درنگ، آینه duty دست‌نخورده)؛ هر دو گیت سبز</t>
         </is>
       </c>
     </row>

</xml_diff>